<commit_message>
Final concentration layout fix
</commit_message>
<xml_diff>
--- a/app/components/ריכוז ספקים.xlsx
+++ b/app/components/ריכוז ספקים.xlsx
@@ -106,8 +106,33 @@
           <t xml:space="preserve">ריכוז ספקים</t>
         </is>
       </c>
-    </row>
-    <row r="2">
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
       <c r="A2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">שם פרויקט</t>
@@ -130,16 +155,16 @@
       </c>
       <c r="E2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">הבטחת איכות</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t xml:space="preserve">תיקו הנדסה אזרחית</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">בקרת איכות</t>
@@ -152,54 +177,74 @@
       </c>
       <c r="C3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">הבטחת איכות</t>
+          <t xml:space="preserve">שם הקבלן</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">תיקו הנדסה אזרחית</t>
+          <t xml:space="preserve">מפלסי הגליל סלילה עפר ופיתוח בע"מ</t>
         </is>
       </c>
       <c r="E3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">מקור נתונים</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">בקרה מקדימה / ספקים</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">מקור נתונים</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">בקרה מקדימה / ספקים</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">שם הקבלן</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">מפלסי הגליל סלילה עפר ופיתוח בע"מ</t>
+      <c r="A4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -556,5 +601,8 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
match all concentration headers to matzea layout
</commit_message>
<xml_diff>
--- a/app/components/ריכוז ספקים.xlsx
+++ b/app/components/ריכוז ספקים.xlsx
@@ -127,7 +127,7 @@
     <col min="9" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">ריכוז ספקים</t>
@@ -164,11 +164,6 @@
         </is>
       </c>
       <c r="H1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -177,7 +172,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">שם פרויקט</t>
+          <t xml:space="preserve">שם פרויקט:</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="2">
@@ -187,173 +182,227 @@
       </c>
       <c r="C2" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">ניהול פרויקט</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="F2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">א. ש. רונן הנדסה אזרחית בע"מ</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">קבלן</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">מפלסי הגליל סלילה עפר ופיתוח בע"מ</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">בקרת איכות</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">קונטרולינג פריים בע"מ</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">שם הקבלן</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">מפלסי הגליל סלילה עפר ופיתוח בע"מ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">הבטחת איכות</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr" s="2">
+      <c r="F3" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">תיקו הנדסה אזרחית</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">מנהל עבודה</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">חוסיין מריסאת</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">מודד</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">באסל אבו שקארה</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">מפקח</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">עאמר והיב</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="10" customHeight="1"/>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" t="inlineStr" s="3">
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">בקרת איכות</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">קונטרולינג פריים בע"מ</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">מקור נתונים</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">בקרה מקדימה / ספקים</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1"/>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">מס׳</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr" s="3">
+      <c r="B6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">שם ספק</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr" s="3">
+      <c r="C6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">חומר/מוצר מסופק</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr" s="3">
+      <c r="D6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">תאריך אישור</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr" s="3">
+      <c r="E6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">מספר תעודה / רישיון / אישור</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr" s="3">
+      <c r="F6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">סוג תעודה /ISO/ת״ת/רישיון</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr" s="3">
+      <c r="G6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">סטטוס</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr" s="3">
+      <c r="H6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">תוקף</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr" s="3">
+      <c r="I6" t="inlineStr" s="3">
         <is>
           <t xml:space="preserve">הערות</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="5">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="6">
         <v>1</v>
       </c>
-      <c r="B6" t="inlineStr" s="5">
+      <c r="B7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">אליהו תעשיות פלסיק בע"מ</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="5">
+      <c r="C7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">מובילי פלסטיק למתקני חשמל ותקשורת</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="5">
+      <c r="D7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">24/04/2026</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr" s="5">
+      <c r="E7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">97252</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr" s="5">
+      <c r="F7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">ISO</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr" s="5">
+      <c r="G7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">מאושר</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr" s="5">
+      <c r="H7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">06/05/2028</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr" s="5">
+      <c r="I7" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+  <mergeCells count="13">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>